<commit_message>
Rev D: correct board order, BOM and review dispositions
</commit_message>
<xml_diff>
--- a/releases/evt-pre-20/2026-09-30-rev-d/Основной_пакет/01_Закупка/BOM_EVT_PRE_20_оценочные_цены.xlsx
+++ b/releases/evt-pre-20/2026-09-30-rev-d/Основной_пакет/01_Закупка/BOM_EVT_PRE_20_оценочные_цены.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка закупки" sheetId="1" r:id="R61a15c257dc34089"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Цены v02" sheetId="2" r:id="R553626595a8841ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DNP" sheetId="3" r:id="Rd67cbfa42ddd486b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка закупки" sheetId="1" r:id="R8e6dd74e9593466f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Цены v02" sheetId="2" r:id="R3ab9c235aaf14899"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DNP" sheetId="3" r:id="Ra463d3fa6d5d4dcd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -671,7 +671,7 @@
         <x:v>DIO-ASM-PWR-REV-A</x:v>
       </x:c>
       <x:c r="H10" s="11" t="str">
-        <x:v>4-layer PCB-PWR Rev A PCBA; JLC04161H-3313A order basis; 90x60x1.6 mm; ENIG; outer 2 oz / 70 um, inner 1 oz / 35 um; fab DFM and actual stack ID at checkout</x:v>
+        <x:v>4-layer PCB-PWR Rev A PCBA; 90x60x1.6 mm; ENIG; 1 oz / 35 um copper on all four layers; fabricator stack ID and DFM at checkout</x:v>
       </x:c>
       <x:c r="I10" s="11" t="str">
         <x:v>N/A</x:v>
@@ -6230,7 +6230,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bb7934a927f4d12"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1b022b46e084a09"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7928,7 +7928,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d63aadd1ce04921"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5aa7df70de6430e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8148,7 +8148,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52e1f29af00242bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re380c74ea45542af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>